<commit_message>
Mudei para michele visualizar
</commit_message>
<xml_diff>
--- a/teste.xlsx
+++ b/teste.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -382,6 +382,14 @@
         <v>6666</v>
       </c>
     </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>25212</v>
+      </c>
+      <c r="B6">
+        <v>255633</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>